<commit_message>
Remove checklist 'Cek No Resi 7-Eleven' and Add feature 'File Name Checking' with keyword 'ELEVEN' and 'FAMI'
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ALL Project\Bikin keterangan Resi\ResiText-App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67E71472-7A4F-4D74-B477-9A3FAC1EFA45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6C5AA8C-49C5-44E5-B8F8-E7E54133C487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2282" yWindow="2282" windowWidth="19563" windowHeight="10162" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,74 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="22">
-  <si>
-    <t>READY</t>
-  </si>
-  <si>
-    <t>3 ODOL MARVIS SILVER</t>
-  </si>
-  <si>
-    <t>6 ELIPS KOMPLIT</t>
-  </si>
-  <si>
-    <t>1 HB M56 + 1 HB GLOSSY</t>
-  </si>
-  <si>
-    <t>3 COLLAGEN COFFEE</t>
-  </si>
-  <si>
-    <t>3 ODOL MARVIS SILVER+3 COLLAGEN COFFEE</t>
-  </si>
-  <si>
-    <t>6 ODOL MARVIS SILVER+3 COLLAGEN COFFEE</t>
-  </si>
-  <si>
-    <t>1 PAKET ISI 4 BRA RENDA HITAM ABU ARMY MERAH 38 + 1 SET CD ACAK</t>
-  </si>
-  <si>
-    <t>1 SMARTWATCH Y13 HITAM + 1 SMARTBAND M8</t>
-  </si>
-  <si>
-    <t>FAMI</t>
-  </si>
-  <si>
-    <t>L25B020T6S</t>
-  </si>
-  <si>
-    <t>L25B020T6T</t>
-  </si>
-  <si>
-    <t>L25B020T6U</t>
-  </si>
-  <si>
-    <t>L25B020T6V</t>
-  </si>
-  <si>
-    <t>L25B020T6W</t>
-  </si>
-  <si>
-    <t>L25B020T6X</t>
-  </si>
-  <si>
-    <t>L25B020T6Y</t>
-  </si>
-  <si>
-    <t>L25B020T6Z</t>
-  </si>
-  <si>
-    <t>L25B020T70</t>
-  </si>
-  <si>
-    <t>L25B020T71</t>
-  </si>
-  <si>
-    <t>L25B020T72</t>
-  </si>
-  <si>
-    <t>L25B020T73</t>
-  </si>
-</sst>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -790,257 +723,113 @@
     <col min="1" max="1" width="26.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28.55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="30" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="31">
-        <v>450</v>
-      </c>
+    <row r="1" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="30"/>
+      <c r="B1" s="31"/>
       <c r="C1" s="32"/>
-      <c r="D1" s="23" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="34" t="s">
-        <v>9</v>
-      </c>
-      <c r="F1" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1" s="35">
-        <v>15320310307</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="28.55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="28" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="29">
-        <v>450</v>
-      </c>
+      <c r="D1" s="23"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="35"/>
+    </row>
+    <row r="2" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="28"/>
+      <c r="B2" s="29"/>
       <c r="C2" s="18"/>
-      <c r="D2" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="36" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="37">
-        <v>15320310305</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="28.55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="28" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="29">
-        <v>390</v>
-      </c>
+      <c r="D2" s="26"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="37"/>
+    </row>
+    <row r="3" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="28"/>
+      <c r="B3" s="29"/>
       <c r="C3" s="18"/>
-      <c r="D3" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="36" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="37">
-        <v>15320310304</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="28.55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="28" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="29">
-        <v>390</v>
-      </c>
+      <c r="D3" s="26"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="37"/>
+    </row>
+    <row r="4" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="28"/>
+      <c r="B4" s="29"/>
       <c r="C4" s="18"/>
-      <c r="D4" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="36" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="20" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="37">
-        <v>15320309533</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="28.55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="28" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="29">
-        <v>390</v>
-      </c>
+      <c r="D4" s="26"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="37"/>
+    </row>
+    <row r="5" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="28"/>
+      <c r="B5" s="29"/>
       <c r="C5" s="18"/>
-      <c r="D5" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="36" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="37">
-        <v>15320309534</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="28.55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="28" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="29">
-        <v>390</v>
-      </c>
+      <c r="D5" s="26"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="37"/>
+    </row>
+    <row r="6" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="28"/>
+      <c r="B6" s="29"/>
       <c r="C6" s="18"/>
-      <c r="D6" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="36" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" s="37">
-        <v>15320309531</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="28.55" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="28" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7" s="29">
-        <v>390</v>
-      </c>
+      <c r="D6" s="26"/>
+      <c r="E6" s="36"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="37"/>
+    </row>
+    <row r="7" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="28"/>
+      <c r="B7" s="29"/>
       <c r="C7" s="18"/>
-      <c r="D7" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="36" t="s">
-        <v>9</v>
-      </c>
-      <c r="F7" s="20" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="37">
-        <v>15320309529</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="33.299999999999997" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="28" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="29">
-        <v>840</v>
-      </c>
+      <c r="D7" s="26"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="37"/>
+    </row>
+    <row r="8" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="28"/>
+      <c r="B8" s="29"/>
       <c r="C8" s="18"/>
-      <c r="D8" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="36" t="s">
-        <v>9</v>
-      </c>
-      <c r="F8" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="G8" s="37">
-        <v>15320310303</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="33.299999999999997" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="28" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="29">
-        <v>1230</v>
-      </c>
+      <c r="D8" s="26"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="37"/>
+    </row>
+    <row r="9" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="28"/>
+      <c r="B9" s="29"/>
       <c r="C9" s="18"/>
-      <c r="D9" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="36" t="s">
-        <v>9</v>
-      </c>
-      <c r="F9" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="G9" s="37">
-        <v>15320309535</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="33.299999999999997" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="25">
-        <v>580</v>
-      </c>
+      <c r="D9" s="26"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="37"/>
+    </row>
+    <row r="10" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="24"/>
+      <c r="B10" s="25"/>
       <c r="C10" s="33"/>
-      <c r="D10" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="E10" s="36" t="s">
-        <v>9</v>
-      </c>
-      <c r="F10" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="G10" s="37">
-        <v>15320310306</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="49.6" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="25">
-        <v>490</v>
-      </c>
+      <c r="D10" s="26"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="38"/>
+      <c r="G10" s="37"/>
+    </row>
+    <row r="11" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="24"/>
+      <c r="B11" s="25"/>
       <c r="C11" s="20"/>
-      <c r="D11" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="E11" s="36" t="s">
-        <v>9</v>
-      </c>
-      <c r="F11" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="G11" s="37">
-        <v>15320309530</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="49.6" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" s="25">
-        <v>499</v>
-      </c>
+      <c r="D11" s="26"/>
+      <c r="E11" s="36"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="37"/>
+    </row>
+    <row r="12" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="24"/>
+      <c r="B12" s="25"/>
       <c r="C12" s="20"/>
-      <c r="D12" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="E12" s="36" t="s">
-        <v>9</v>
-      </c>
-      <c r="F12" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="G12" s="39">
-        <v>15320309532</v>
-      </c>
+      <c r="D12" s="26"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="39"/>
     </row>
     <row r="13" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="24"/>

</xml_diff>